<commit_message>
Update schedule milestones and specify three required sabikan training certificates.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/public/downloads/opening-schedule.xlsx
+++ b/docs/public/downloads/opening-schedule.xlsx
@@ -73,19 +73,19 @@
     <t>利用者募集の準備開始（パンフレット案・見学導線）</t>
   </si>
   <si>
+    <t>指定申請に必要な資料の準備（上位店の指示に従う）</t>
+  </si>
+  <si>
     <t>60日前</t>
   </si>
   <si>
     <t>サビ管の雇用条件合意・勤務開始日調整</t>
   </si>
   <si>
-    <t>物件の最終選定結果を上位店から確認</t>
+    <t>物件の最終選定結果を上位店へ報告</t>
   </si>
   <si>
     <t>主要職員（管理者・生援・職指）の採用決定</t>
-  </si>
-  <si>
-    <t>指定申請に必要な資料の準備（上位店の指示に従う）</t>
   </si>
   <si>
     <t>IT環境整備開始（HP・SNS・電話・メール）</t>
@@ -807,26 +807,26 @@
         <v>19</v>
       </c>
     </row>
-    <row r="22" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A22" s="2" t="s">
+    <row r="21" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="B21" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="2"/>
-    </row>
-    <row r="23" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A23" s="3" t="s">
+    </row>
+    <row r="23" ht="24" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B23" s="2"/>
+    </row>
+    <row r="24" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="B23" s="3" t="s">
+      <c r="B24" s="3" t="s">
         <v>3</v>
-      </c>
-    </row>
-    <row r="24" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A24" s="4" t="s">
-        <v>4</v>
-      </c>
-      <c r="B24" s="5" t="s">
-        <v>21</v>
       </c>
     </row>
     <row r="25" ht="20" customHeight="1" spans="1:2" x14ac:dyDescent="0.25">
@@ -1224,7 +1224,7 @@
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="A2:B2"/>
     <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
     <mergeCell ref="A32:B32"/>
     <mergeCell ref="A38:B38"/>
     <mergeCell ref="A51:B51"/>

</xml_diff>